<commit_message>
update template lich tiep dan
</commit_message>
<xml_diff>
--- a/src/public/static/template-lich-tiep-dan.xlsx
+++ b/src/public/static/template-lich-tiep-dan.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11460"/>
+    <workbookView windowWidth="21375" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Địa điểm</t>
   </si>
@@ -35,24 +35,24 @@
     <t>Tên cán bộ</t>
   </si>
   <si>
-    <t>Thời gian</t>
-  </si>
-  <si>
     <t>Ngày tiếp dân</t>
   </si>
   <si>
     <t>Ghi chú</t>
   </si>
   <si>
+    <t>Từ</t>
+  </si>
+  <si>
+    <t>Đến</t>
+  </si>
+  <si>
     <t>P.001</t>
   </si>
   <si>
     <t>Lê Văn A</t>
   </si>
   <si>
-    <t>03:00 - 10:00</t>
-  </si>
-  <si>
     <t>Truc tiep</t>
   </si>
   <si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>Nguyễn Thị H</t>
-  </si>
-  <si>
-    <t>08:00 - 10:00</t>
   </si>
   <si>
     <t>Online</t>
@@ -84,12 +81,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="m/d/yyyy;@"/>
+    <numFmt numFmtId="179" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -694,11 +692,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
@@ -1237,17 +1238,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="4"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="17.4285714285714" customWidth="1"/>
-    <col min="2" max="2" width="27.4285714285714" customWidth="1"/>
-    <col min="3" max="3" width="25.1428571428571" customWidth="1"/>
-    <col min="4" max="4" width="16.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="2" max="2" width="17.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="16.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="13.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="17.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="16.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1263,71 +1265,89 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
+      <c r="C2" s="1">
         <v>45931</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
+      <c r="E2" s="2">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.333333333333333</v>
+      </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1">
+        <v>45932</v>
+      </c>
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="2">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3">
         <v>45932</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3">
         <v>45932</v>
       </c>
-      <c r="E4" t="s">
-        <v>12</v>
+      <c r="E5" s="2">
+        <v>0.958333333333333</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2">
-        <v>45932</v>
-      </c>
+    <row r="6" spans="5:5">
+      <c r="E6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add executable reception swagger demos
</commit_message>
<xml_diff>
--- a/src/public/static/template-lich-tiep-dan.xlsx
+++ b/src/public/static/template-lich-tiep-dan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>Địa điểm</t>
   </si>
@@ -35,10 +35,10 @@
     <t>Bộ phận tiếp công dân</t>
   </si>
   <si>
-    <t>Nguyễn Văn An</t>
-  </si>
-  <si>
-    <t>25/08/2026</t>
+    <t>Cán bộ Swagger Import Sáng</t>
+  </si>
+  <si>
+    <t>01/09/2099</t>
   </si>
   <si>
     <t>Ca buổi sáng</t>
@@ -50,7 +50,10 @@
     <t>11:30</t>
   </si>
   <si>
-    <t>Trần Thị Bình</t>
+    <t>Cán bộ Swagger Import Chiều</t>
+  </si>
+  <si>
+    <t>02/09/2099</t>
   </si>
   <si>
     <t>Ca buổi chiều</t>
@@ -554,16 +557,16 @@
         <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -584,18 +587,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -603,39 +606,39 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -643,7 +646,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>